<commit_message>
add morgan abalation result
</commit_message>
<xml_diff>
--- a/abalation/main_text_ablation_table.xlsx
+++ b/abalation/main_text_ablation_table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,80 +473,120 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Random selection</t>
+          <t>Full model</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>647</v>
+        <v>70</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.5217 ± 0.1478</t>
+          <t>0.7907 ± 0.0300</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>7/7</t>
+          <t>5/7</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.5297</t>
+          <t>0.7229</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.7775</t>
+          <t>0.8904</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2.1006%</t>
+          <t>0.2273%</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0.5965</t>
+          <t>0.9762</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Full model</t>
+          <t>Random selection</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>70</v>
+        <v>647</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.7907 ± 0.0300</t>
+          <t>0.5217 ± 0.1478</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5/7</t>
+          <t>7/7</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.7229</t>
+          <t>0.5297</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.8904</t>
+          <t>0.7775</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0.2273%</t>
+          <t>2.1006%</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>0.9762</t>
+          <t>0.5965</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Morgan fingerprints</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1598</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0.4971 ± 0.1772</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>7/7</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.8369</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.7417</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>5.1883%</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0.4084</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add radar for ablation
</commit_message>
<xml_diff>
--- a/abalation/main_text_ablation_table.xlsx
+++ b/abalation/main_text_ablation_table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,15 +456,30 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Known-additive similarity</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Novelty score ↑</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Moderate novelty ratio</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Candidate diversity ↑</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Post-screening survival ↑</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Silhouette ↑</t>
         </is>
@@ -477,11 +492,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.7907 ± 0.0300</t>
+          <t>0.7898 ± 0.0306</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -491,22 +506,37 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.7229</t>
+          <t>0.7232</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.8904</t>
+          <t>0.4025 ± 0.2446</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.2273%</t>
+          <t>0.5975 ± 0.2446</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0.9762</t>
+          <t>25.35%</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0.8982</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0.2305%</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>0.9761</t>
         </is>
       </c>
     </row>
@@ -536,15 +566,30 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.7775</t>
+          <t>0.3565 ± 0.0910</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>0.6435 ± 0.0910</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>24.42%</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0.7830</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>2.1006%</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>0.5965</t>
         </is>
@@ -576,15 +621,30 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.7417</t>
+          <t>0.3696 ± 0.0875</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>0.6304 ± 0.0875</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>29.10%</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0.7474</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>5.1883%</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>0.4084</t>
         </is>
@@ -597,11 +657,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1745</v>
+        <v>573</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.1410 ± 0.0453</t>
+          <t>0.1413 ± 0.0366</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -611,22 +671,37 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.8897</t>
+          <t>0.6693</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.8933</t>
+          <t>0.3278 ± 0.1029</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5.6656%</t>
+          <t>0.6722 ± 0.1029</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0.4581</t>
+          <t>12.91%</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0.8101</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1.8604%</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>0.2533</t>
         </is>
       </c>
     </row>
@@ -637,36 +712,51 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2853</v>
+        <v>1741</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.0958 ± 0.0377</t>
+          <t>0.0807 ± 0.0149</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6/7</t>
+          <t>4/7</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.3038</t>
+          <t>0.0371</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.8280</t>
+          <t>0.3730 ± 0.0817</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>9.2630%</t>
+          <t>0.6270 ± 0.0817</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>-0.2067</t>
+          <t>30.21%</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0.7338</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>5.6526%</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>-0.2245</t>
         </is>
       </c>
     </row>
@@ -677,7 +767,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1065</v>
+        <v>297</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -696,15 +786,30 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0.8677</t>
+          <t>0.3442 ± 0.2060</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3.4578%</t>
+          <t>0.6558 ± 0.2060</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
+        <is>
+          <t>23.91%</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0.8660</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>0.9643%</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>nan</t>
         </is>

</xml_diff>